<commit_message>
Adding additional comments about the hydo peaking
</commit_message>
<xml_diff>
--- a/InputData/elec/BPaFF/Boolean Peaking and Flexibility Flags.xlsx
+++ b/InputData/elec/BPaFF/Boolean Peaking and Flexibility Flags.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="4245" yWindow="2430" windowWidth="17280" windowHeight="9960" activeTab="2"/>
+    <workbookView xWindow="4245" yWindow="2430" windowWidth="17280" windowHeight="9960"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="47">
   <si>
     <t>Source:</t>
   </si>
@@ -172,13 +172,38 @@
   </si>
   <si>
     <t>Using [eps-brazil-2.1.1] values in both tables</t>
+  </si>
+  <si>
+    <r>
+      <t>CPL’s research found that hydro provides both load-following and flexibility for Brazil’s grid, so we concluded the value of  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  for both flags.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,6 +214,20 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -215,12 +254,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -525,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -554,118 +594,124 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="C7" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>